<commit_message>
changed the nav data and metrics from 31 jul 25 - 31 jul 26
</commit_message>
<xml_diff>
--- a/algorithm/output_result/category_comparision/Category_Comparison.xlsx
+++ b/algorithm/output_result/category_comparision/Category_Comparison.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,10 +531,10 @@
         <v>67</v>
       </c>
       <c r="H3" t="n">
-        <v>65.33</v>
+        <v>67</v>
       </c>
       <c r="I3" t="n">
-        <v>59.7</v>
+        <v>60.2</v>
       </c>
     </row>
     <row r="4">
@@ -595,20 +595,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Top 300 Alpha 50 Fund</t>
+          <t>Discovery Fund</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>92.31</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="H5" t="n">
-        <v>57.33</v>
+        <v>69.67</v>
       </c>
       <c r="I5" t="n">
-        <v>82.02</v>
+        <v>80.7</v>
       </c>
     </row>
     <row r="6">
@@ -632,20 +632,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Discovery Fund</t>
+          <t>Top 300 Alpha 50 Fund</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>84.62</v>
       </c>
       <c r="G6" t="n">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="H6" t="n">
-        <v>68</v>
+        <v>57.33</v>
       </c>
       <c r="I6" t="n">
-        <v>80.2</v>
+        <v>78.95</v>
       </c>
     </row>
     <row r="7">
@@ -669,20 +669,20 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Opportunities Fund</t>
+          <t>India Consumption Advantage Fund</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>84.62</v>
+        <v>76.92</v>
       </c>
       <c r="G7" t="n">
-        <v>61</v>
+        <v>95</v>
       </c>
       <c r="H7" t="n">
-        <v>59.67</v>
+        <v>50.28</v>
       </c>
       <c r="I7" t="n">
-        <v>70.05</v>
+        <v>74.34999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -706,20 +706,20 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>India Consumption Advantage Fund</t>
+          <t>Opportunities Fund</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>61.54</v>
+        <v>92.31</v>
       </c>
       <c r="G8" t="n">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="H8" t="n">
-        <v>50.28</v>
+        <v>59.67</v>
       </c>
       <c r="I8" t="n">
-        <v>68.2</v>
+        <v>73.12</v>
       </c>
     </row>
     <row r="9">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>38.46</v>
+        <v>46.15</v>
       </c>
       <c r="G9" t="n">
         <v>88</v>
@@ -756,7 +756,7 @@
         <v>56.67</v>
       </c>
       <c r="I9" t="n">
-        <v>58.78</v>
+        <v>61.86</v>
       </c>
     </row>
     <row r="10">
@@ -780,20 +780,20 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>India Sector Leaders Opportunities Fund</t>
+          <t>Sustainable Equity Fund</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>69.23</v>
+        <v>53.85</v>
       </c>
       <c r="G10" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I10" t="n">
-        <v>57.69</v>
+        <v>60.54</v>
       </c>
     </row>
     <row r="11">
@@ -817,20 +817,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nifty Alpha 30 Fund</t>
+          <t>Top 500 Multifactor 50 Fund</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>76.92</v>
+        <v>30.77</v>
       </c>
       <c r="G11" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="H11" t="n">
-        <v>56.33</v>
+        <v>50</v>
       </c>
       <c r="I11" t="n">
-        <v>53.67</v>
+        <v>56.71</v>
       </c>
     </row>
     <row r="12">
@@ -854,20 +854,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Top 500 Multifactor 50 Fund</t>
+          <t>India Sector Leaders Opportunities Fund</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>23.08</v>
+        <v>61.54</v>
       </c>
       <c r="G12" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H12" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>52.43</v>
+        <v>54.62</v>
       </c>
     </row>
     <row r="13">
@@ -891,20 +891,20 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sustainable Equity Fund</t>
+          <t>Nifty Alpha 30 Fund</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>30.77</v>
+        <v>69.23</v>
       </c>
       <c r="G13" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="H13" t="n">
-        <v>50</v>
+        <v>56.33</v>
       </c>
       <c r="I13" t="n">
-        <v>51.31</v>
+        <v>50.59</v>
       </c>
     </row>
     <row r="14">
@@ -928,20 +928,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Midcap Momentum Fund</t>
+          <t>Equity Advantage Fund</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>53.85</v>
+        <v>23.08</v>
       </c>
       <c r="G14" t="n">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="H14" t="n">
-        <v>50.67</v>
+        <v>58.33</v>
       </c>
       <c r="I14" t="n">
-        <v>50.54</v>
+        <v>48.63</v>
       </c>
     </row>
     <row r="15">
@@ -965,20 +965,20 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Top 500 Momentum 50 Fund</t>
+          <t>Diversified Equity Fund</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>46.15</v>
+        <v>7.69</v>
       </c>
       <c r="G15" t="n">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="H15" t="n">
-        <v>63</v>
+        <v>58.33</v>
       </c>
       <c r="I15" t="n">
-        <v>49.06</v>
+        <v>45.47</v>
       </c>
     </row>
     <row r="16">
@@ -1002,20 +1002,20 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Diversified Equity Fund</t>
+          <t>Midcap Momentum Fund</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>7.69</v>
+        <v>38.46</v>
       </c>
       <c r="G16" t="n">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="H16" t="n">
-        <v>60</v>
+        <v>52.33</v>
       </c>
       <c r="I16" t="n">
-        <v>45.98</v>
+        <v>44.88</v>
       </c>
     </row>
     <row r="17">
@@ -1039,20 +1039,20 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Equity Advantage Fund</t>
+          <t>Blue Chip Fund</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>15.38</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="H17" t="n">
-        <v>58.33</v>
+        <v>56.67</v>
       </c>
       <c r="I17" t="n">
-        <v>45.55</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="18">
@@ -1076,20 +1076,20 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Blue Chip Fund</t>
+          <t>Top 500 Momentum 50 Fund</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>15.38</v>
       </c>
       <c r="G18" t="n">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="H18" t="n">
-        <v>56.67</v>
+        <v>59.67</v>
       </c>
       <c r="I18" t="n">
-        <v>42.5</v>
+        <v>35.75</v>
       </c>
     </row>
     <row r="19">
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G19" t="n">
         <v>100</v>
@@ -1126,7 +1126,7 @@
         <v>68</v>
       </c>
       <c r="I19" t="n">
-        <v>90.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1163,7 +1163,7 @@
         <v>55</v>
       </c>
       <c r="I20" t="n">
-        <v>36.5</v>
+        <v>56.5</v>
       </c>
     </row>
     <row r="21">
@@ -1228,16 +1228,16 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>81.48</v>
+        <v>95.83</v>
       </c>
       <c r="G22" t="n">
         <v>56</v>
       </c>
       <c r="H22" t="n">
-        <v>68</v>
+        <v>61.33</v>
       </c>
       <c r="I22" t="n">
-        <v>69.79000000000001</v>
+        <v>73.53</v>
       </c>
     </row>
     <row r="23">
@@ -1261,20 +1261,20 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mid Cap Fund</t>
+          <t>Maximise India Fund</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>92.59</v>
+        <v>70.83</v>
       </c>
       <c r="G23" t="n">
-        <v>7</v>
+        <v>68</v>
       </c>
       <c r="H23" t="n">
-        <v>86.67</v>
+        <v>58.33</v>
       </c>
       <c r="I23" t="n">
-        <v>65.14</v>
+        <v>66.23</v>
       </c>
     </row>
     <row r="24">
@@ -1298,20 +1298,20 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Nifty Alpha 50 Index Fund</t>
+          <t>MidSmallCap 400 Momentum Quality 100 Index Fund</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>100</v>
+        <v>79.17</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="H24" t="n">
-        <v>76.67</v>
+        <v>54.67</v>
       </c>
       <c r="I24" t="n">
-        <v>63.6</v>
+        <v>63.37</v>
       </c>
     </row>
     <row r="25">
@@ -1335,20 +1335,20 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Mid Cap Index Fund</t>
+          <t>Multicap 50 25 25 Index Fund</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>88.89</v>
+        <v>66.67</v>
       </c>
       <c r="G25" t="n">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="H25" t="n">
-        <v>86.67</v>
+        <v>55</v>
       </c>
       <c r="I25" t="n">
-        <v>63.06</v>
+        <v>62.07</v>
       </c>
     </row>
     <row r="26">
@@ -1372,20 +1372,20 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Value Enhancer Fund</t>
+          <t>Mid Cap Fund</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>85.19</v>
+        <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H26" t="n">
-        <v>83.33</v>
+        <v>66.33</v>
       </c>
       <c r="I26" t="n">
-        <v>62.08</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27">
@@ -1409,20 +1409,20 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Maximise India Fund</t>
+          <t>Smallcap250 Momentum Quality 100 Index Fund</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>55.56</v>
+        <v>91.67</v>
       </c>
       <c r="G27" t="n">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="H27" t="n">
-        <v>63.33</v>
+        <v>50.67</v>
       </c>
       <c r="I27" t="n">
-        <v>61.62</v>
+        <v>59.07</v>
       </c>
     </row>
     <row r="28">
@@ -1446,20 +1446,20 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Multicap 50 25 25 Index Fund</t>
+          <t>Value Enhancer Fund</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>48.15</v>
+        <v>87.5</v>
       </c>
       <c r="G28" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="H28" t="n">
-        <v>63.33</v>
+        <v>64.67</v>
       </c>
       <c r="I28" t="n">
-        <v>57.16</v>
+        <v>57.4</v>
       </c>
     </row>
     <row r="29">
@@ -1483,20 +1483,20 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Smallcap250 Momentum Quality 100 Index Fund</t>
+          <t>Pension Opportunities Fund</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>77.78</v>
+        <v>58.33</v>
       </c>
       <c r="G29" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="H29" t="n">
-        <v>62.33</v>
+        <v>63.33</v>
       </c>
       <c r="I29" t="n">
-        <v>57.01</v>
+        <v>54.63</v>
       </c>
     </row>
     <row r="30">
@@ -1520,20 +1520,20 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Multi Cap Growth Fund</t>
+          <t>India Consumption Fund</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>70.37</v>
+        <v>83.33</v>
       </c>
       <c r="G30" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H30" t="n">
-        <v>66.67</v>
+        <v>46.67</v>
       </c>
       <c r="I30" t="n">
-        <v>56.25</v>
+        <v>50.93</v>
       </c>
     </row>
     <row r="31">
@@ -1557,20 +1557,20 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pension Opportunities Fund</t>
+          <t>Pension India Growth Fund</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>62.96</v>
+        <v>45.83</v>
       </c>
       <c r="G31" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H31" t="n">
-        <v>60</v>
+        <v>58.33</v>
       </c>
       <c r="I31" t="n">
-        <v>55.48</v>
+        <v>49.03</v>
       </c>
     </row>
     <row r="32">
@@ -1594,20 +1594,20 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Opportunities Fund</t>
+          <t>Pension India Consumption Fund</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>66.67</v>
+        <v>75</v>
       </c>
       <c r="G32" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="H32" t="n">
-        <v>56.67</v>
+        <v>46.67</v>
       </c>
       <c r="I32" t="n">
-        <v>54.77</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="33">
@@ -1631,20 +1631,20 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Smallcap 250 Index Fund</t>
+          <t>Opportunities Fund</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>96.3</v>
+        <v>41.67</v>
       </c>
       <c r="G33" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I33" t="n">
-        <v>54.72</v>
+        <v>45.77</v>
       </c>
     </row>
     <row r="34">
@@ -1668,20 +1668,20 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pension India Growth Fund</t>
+          <t>Sustainable Equity Fund</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>59.26</v>
+        <v>50</v>
       </c>
       <c r="G34" t="n">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="H34" t="n">
-        <v>56.67</v>
+        <v>51.67</v>
       </c>
       <c r="I34" t="n">
-        <v>53.9</v>
+        <v>45.1</v>
       </c>
     </row>
     <row r="35">
@@ -1709,16 +1709,16 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>74.06999999999999</v>
+        <v>54.17</v>
       </c>
       <c r="G35" t="n">
         <v>17</v>
       </c>
       <c r="H35" t="n">
-        <v>63.33</v>
+        <v>58.33</v>
       </c>
       <c r="I35" t="n">
-        <v>53.73</v>
+        <v>44.27</v>
       </c>
     </row>
     <row r="36">
@@ -1742,20 +1742,20 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>MidSmallCap 400 Momentum Quality 100 Index Fund</t>
+          <t>Bluechip Fund</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>33.33</v>
+        <v>16.67</v>
       </c>
       <c r="G36" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="H36" t="n">
-        <v>61.33</v>
+        <v>53.33</v>
       </c>
       <c r="I36" t="n">
-        <v>47.03</v>
+        <v>43.97</v>
       </c>
     </row>
     <row r="37">
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>18.52</v>
+        <v>12.5</v>
       </c>
       <c r="G37" t="n">
         <v>76</v>
@@ -1792,7 +1792,7 @@
         <v>53.33</v>
       </c>
       <c r="I37" t="n">
-        <v>46.21</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="38">
@@ -1816,20 +1816,20 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Bluechip Fund</t>
+          <t>Mid Cap 150 Momentum 50 Index Fund</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>22.22</v>
+        <v>37.5</v>
       </c>
       <c r="G38" t="n">
-        <v>71</v>
+        <v>34</v>
       </c>
       <c r="H38" t="n">
-        <v>53.33</v>
+        <v>54.67</v>
       </c>
       <c r="I38" t="n">
-        <v>46.19</v>
+        <v>41.6</v>
       </c>
     </row>
     <row r="39">
@@ -1857,16 +1857,16 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>11.11</v>
+        <v>8.33</v>
       </c>
       <c r="G39" t="n">
         <v>78</v>
       </c>
       <c r="H39" t="n">
-        <v>51.67</v>
+        <v>48.33</v>
       </c>
       <c r="I39" t="n">
-        <v>43.34</v>
+        <v>41.23</v>
       </c>
     </row>
     <row r="40">
@@ -1890,20 +1890,20 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>India Consumption Fund</t>
+          <t>Smallcap 250 Index Fund</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>51.85</v>
+        <v>62.5</v>
       </c>
       <c r="G40" t="n">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="H40" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>42.34</v>
+        <v>41.2</v>
       </c>
     </row>
     <row r="41">
@@ -1927,20 +1927,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sector Leaders Index Fund</t>
+          <t>Multi Cap Growth Fund</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>29.63</v>
+        <v>33.33</v>
       </c>
       <c r="G41" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="H41" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="I41" t="n">
-        <v>41.55</v>
+        <v>37.93</v>
       </c>
     </row>
     <row r="42">
@@ -1964,20 +1964,20 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pension India Consumption Fund</t>
+          <t>India Growth Fund</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>44.44</v>
+        <v>29.17</v>
       </c>
       <c r="G42" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H42" t="n">
-        <v>60</v>
+        <v>58.33</v>
       </c>
       <c r="I42" t="n">
-        <v>40.28</v>
+        <v>37.87</v>
       </c>
     </row>
     <row r="43">
@@ -2001,20 +2001,20 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>India Growth Fund</t>
+          <t>Sector Leaders Index Fund</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.74</v>
+        <v>20.83</v>
       </c>
       <c r="G43" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="H43" t="n">
-        <v>50</v>
+        <v>44.57</v>
       </c>
       <c r="I43" t="n">
-        <v>40</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="44">
@@ -2042,16 +2042,16 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>37.04</v>
+        <v>25</v>
       </c>
       <c r="G44" t="n">
         <v>24</v>
       </c>
       <c r="H44" t="n">
-        <v>56.67</v>
+        <v>55</v>
       </c>
       <c r="I44" t="n">
-        <v>39.02</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="45">
@@ -2075,20 +2075,20 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mid Cap 150 Momentum 50 Index Fund</t>
+          <t>Dividend Leaders 50 Index Fund</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>14.81</v>
+        <v>4.17</v>
       </c>
       <c r="G45" t="n">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="H45" t="n">
-        <v>61.33</v>
+        <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>34.52</v>
+        <v>19.37</v>
       </c>
     </row>
     <row r="46">
@@ -2112,100 +2112,100 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Sustainable Equity Fund</t>
+          <t>BSE 500 Enhanced Value 50 Index Fund</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>25.93</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>43.33</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>32.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ICICI Prudential</t>
+          <t>Tata AIA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Debt</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Debt - Short Term</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Dividend Leaders 50 Index Fund</t>
+          <t>Whole Life Short-Term Fixed Income Fund</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>3.7</v>
+        <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>86.67</v>
       </c>
       <c r="I47" t="n">
-        <v>19.18</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ICICI Prudential</t>
+          <t>Tata AIA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Debt</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Debt</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BSE 500 Enhanced Value 50 Index Fund</t>
+          <t>Whole Life Income Fund</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>7.41</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>70.33</v>
       </c>
       <c r="I48" t="n">
-        <v>2.96</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ICICI Prudential</t>
+          <t>Tata AIA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2215,23 +2215,29 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+          <t>Equity - Small Cap</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Large N Mid Cap Advantage Fund</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>Small Cap Discovery Fund</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>100</v>
+      </c>
       <c r="G49" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" t="inlineStr"/>
+        <v>69.67</v>
+      </c>
+      <c r="I49" t="n">
+        <v>90.90000000000001</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2241,33 +2247,33 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Debt</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Debt</t>
+          <t>Equity - Mid Cap Oriented</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Whole Life Income Fund</t>
+          <t>Emerging Opportunities Fund</t>
         </is>
       </c>
       <c r="F50" t="n">
+        <v>94.12</v>
+      </c>
+      <c r="G50" t="n">
         <v>100</v>
       </c>
-      <c r="G50" t="n">
-        <v>0</v>
-      </c>
       <c r="H50" t="n">
-        <v>70.33</v>
+        <v>64.67</v>
       </c>
       <c r="I50" t="n">
-        <v>61.1</v>
+        <v>87.05</v>
       </c>
     </row>
     <row r="51">
@@ -2278,33 +2284,33 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Debt</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Debt - Short Term</t>
+          <t>Equity - Thematic (Growth/Domestic)</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Whole Life Short-Term Fixed Income Fund</t>
+          <t>Rising India Fund</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="G51" t="n">
         <v>100</v>
       </c>
       <c r="H51" t="n">
-        <v>86.67</v>
+        <v>62.33</v>
       </c>
       <c r="I51" t="n">
-        <v>56</v>
+        <v>81.64</v>
       </c>
     </row>
     <row r="52">
@@ -2320,28 +2326,28 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Equity - Small Cap</t>
+          <t>Equity - Flexi Cap</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Small Cap Discovery Fund</t>
+          <t>Flexi Growth Fund</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>100</v>
+        <v>76.47</v>
       </c>
       <c r="G52" t="n">
         <v>100</v>
       </c>
       <c r="H52" t="n">
-        <v>69.67</v>
+        <v>59.67</v>
       </c>
       <c r="I52" t="n">
-        <v>90.90000000000001</v>
+        <v>78.48999999999999</v>
       </c>
     </row>
     <row r="53">
@@ -2357,28 +2363,28 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Equity - Mid Cap Oriented</t>
+          <t>Equity - Index (Nifty Alpha 50)</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Emerging Opportunities Fund</t>
+          <t>Nifty Alpha 50 Index Fund</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>94.44</v>
+        <v>70.59</v>
       </c>
       <c r="G53" t="n">
         <v>100</v>
       </c>
       <c r="H53" t="n">
-        <v>64.67</v>
+        <v>54</v>
       </c>
       <c r="I53" t="n">
-        <v>87.18000000000001</v>
+        <v>74.44</v>
       </c>
     </row>
     <row r="54">
@@ -2394,28 +2400,28 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Equity - Thematic (Growth/Domestic)</t>
+          <t>Equity - Large &amp; Mid Cap (BSE 200 oriented)</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Rising India Fund</t>
+          <t>Top 200 Fund</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>77.78</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="G54" t="n">
         <v>100</v>
       </c>
       <c r="H54" t="n">
-        <v>62.33</v>
+        <v>57.33</v>
       </c>
       <c r="I54" t="n">
-        <v>79.81</v>
+        <v>73.08</v>
       </c>
     </row>
     <row r="55">
@@ -2431,28 +2437,28 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Equity - Index (Nifty Alpha 50)</t>
+          <t>Equity - Thematic (Consumption)</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Nifty Alpha 50 Index Fund</t>
+          <t>Tax Bonanza Consumption Fund</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>83.33</v>
+        <v>58.82</v>
       </c>
       <c r="G55" t="n">
         <v>100</v>
       </c>
       <c r="H55" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I55" t="n">
-        <v>79.53</v>
+        <v>68.53</v>
       </c>
     </row>
     <row r="56">
@@ -2468,28 +2474,28 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Equity - Large &amp; Mid Cap (BSE 200 oriented)</t>
+          <t>Equity - Index (Momentum 50)</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Top 200 Fund</t>
+          <t>Momentum 50 Index Fund</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>72.22</v>
+        <v>47.06</v>
       </c>
       <c r="G56" t="n">
         <v>100</v>
       </c>
       <c r="H56" t="n">
-        <v>57.33</v>
+        <v>63.03</v>
       </c>
       <c r="I56" t="n">
-        <v>76.09</v>
+        <v>67.73</v>
       </c>
     </row>
     <row r="57">
@@ -2505,28 +2511,28 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Equity - Multi Cap</t>
+          <t>Equity - Ethical/Exclusionary</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Multi Cap Fund</t>
+          <t>Super Select Equity Fund</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>66.67</v>
+        <v>52.94</v>
       </c>
       <c r="G57" t="n">
         <v>100</v>
       </c>
       <c r="H57" t="n">
-        <v>59.67</v>
+        <v>46.67</v>
       </c>
       <c r="I57" t="n">
-        <v>74.56999999999999</v>
+        <v>65.18000000000001</v>
       </c>
     </row>
     <row r="58">
@@ -2542,28 +2548,28 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Equity - Flexi Cap</t>
+          <t>Balanced - Equity Oriented</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Flexi Growth Fund</t>
+          <t>Whole Life Aggressive Growth Fund</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>61.11</v>
+        <v>41.18</v>
       </c>
       <c r="G58" t="n">
         <v>100</v>
       </c>
       <c r="H58" t="n">
-        <v>59.67</v>
+        <v>59</v>
       </c>
       <c r="I58" t="n">
-        <v>72.34</v>
+        <v>64.17</v>
       </c>
     </row>
     <row r="59">
@@ -2579,28 +2585,28 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Equity - Index (Momentum 50)</t>
+          <t>Equity - Large Cap (Nifty 50 oriented)</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Momentum 50 Index Fund</t>
+          <t>Top 50 Fund</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>50</v>
+        <v>29.41</v>
       </c>
       <c r="G59" t="n">
         <v>100</v>
       </c>
       <c r="H59" t="n">
-        <v>63.03</v>
+        <v>59</v>
       </c>
       <c r="I59" t="n">
-        <v>68.91</v>
+        <v>59.46</v>
       </c>
     </row>
     <row r="60">
@@ -2616,28 +2622,28 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Equity - Thematic (Consumption)</t>
+          <t>Equity - ESG/Thematic</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Tax Bonanza Consumption Fund</t>
+          <t>Sustainable Equity Fund</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>55.56</v>
+        <v>35.29</v>
       </c>
       <c r="G60" t="n">
         <v>100</v>
       </c>
       <c r="H60" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I60" t="n">
-        <v>67.22</v>
+        <v>57.62</v>
       </c>
     </row>
     <row r="61">
@@ -2653,28 +2659,28 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Balanced - Equity Oriented</t>
+          <t>Equity - Large Cap</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Whole Life Aggressive Growth Fund</t>
+          <t>Large Cap Equity Fund</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>38.89</v>
+        <v>23.53</v>
       </c>
       <c r="G61" t="n">
         <v>100</v>
       </c>
       <c r="H61" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I61" t="n">
-        <v>63.26</v>
+        <v>55.61</v>
       </c>
     </row>
     <row r="62">
@@ -2690,28 +2696,28 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Equity - Ethical/Exclusionary</t>
+          <t>Equity - Thematic (Consumption)</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Super Select Equity Fund</t>
+          <t>India Consumption Fund</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>44.44</v>
+        <v>88.23999999999999</v>
       </c>
       <c r="G62" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>46.67</v>
+        <v>64.67</v>
       </c>
       <c r="I62" t="n">
-        <v>61.78</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="63">
@@ -2731,7 +2737,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2739,7 +2745,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>27.78</v>
+        <v>17.65</v>
       </c>
       <c r="G63" t="n">
         <v>100</v>
@@ -2748,7 +2754,7 @@
         <v>55</v>
       </c>
       <c r="I63" t="n">
-        <v>57.61</v>
+        <v>53.56</v>
       </c>
     </row>
     <row r="64">
@@ -2764,28 +2770,28 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Equity - ESG/Thematic</t>
+          <t>Equity - Index (Midcap Momentum)</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Sustainable Equity Fund</t>
+          <t>Midcap Momentum Index Fund</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>33.33</v>
+        <v>5.88</v>
       </c>
       <c r="G64" t="n">
         <v>100</v>
       </c>
       <c r="H64" t="n">
-        <v>45</v>
+        <v>54.67</v>
       </c>
       <c r="I64" t="n">
-        <v>56.83</v>
+        <v>48.75</v>
       </c>
     </row>
     <row r="65">
@@ -2801,28 +2807,28 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Equity - Index (Midcap Momentum)</t>
+          <t>Equity - Index (Sector Leaders)</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Midcap Momentum Index Fund</t>
+          <t>Sector Leaders Index Fund</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>22.22</v>
+        <v>11.76</v>
       </c>
       <c r="G65" t="n">
         <v>100</v>
       </c>
       <c r="H65" t="n">
-        <v>54.67</v>
+        <v>38.86</v>
       </c>
       <c r="I65" t="n">
-        <v>55.29</v>
+        <v>46.36</v>
       </c>
     </row>
     <row r="66">
@@ -2838,28 +2844,28 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Equity - Thematic (Consumption)</t>
+          <t>Equity - Index (Multicap Momentum Quality)</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>India Consumption Fund</t>
+          <t>Multicap Momentum Quality Index Fund</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>88.89</v>
+        <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H66" t="n">
-        <v>64.67</v>
+        <v>49</v>
       </c>
       <c r="I66" t="n">
-        <v>54.96</v>
+        <v>44.7</v>
       </c>
     </row>
     <row r="67">
@@ -2870,180 +2876,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Equity - Large Cap (Nifty 50 oriented)</t>
+          <t>Balanced - Debt Oriented</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Top 50 Fund</t>
+          <t>Whole Life Stable Growth Fund</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>16.67</v>
+        <v>100</v>
       </c>
       <c r="G67" t="n">
         <v>100</v>
       </c>
       <c r="H67" t="n">
-        <v>59</v>
+        <v>64.67</v>
       </c>
       <c r="I67" t="n">
-        <v>54.37</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Tata AIA</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Equity - Large Cap</t>
-        </is>
-      </c>
-      <c r="D68" t="n">
-        <v>17</v>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Large Cap Equity Fund</t>
-        </is>
-      </c>
-      <c r="F68" t="n">
-        <v>11.11</v>
-      </c>
-      <c r="G68" t="n">
-        <v>100</v>
-      </c>
-      <c r="H68" t="n">
-        <v>54</v>
-      </c>
-      <c r="I68" t="n">
-        <v>50.64</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Tata AIA</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Equity - Index (Multicap Momentum Quality)</t>
-        </is>
-      </c>
-      <c r="D69" t="n">
-        <v>18</v>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Multicap Momentum Quality Index Fund</t>
-        </is>
-      </c>
-      <c r="F69" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" t="n">
-        <v>100</v>
-      </c>
-      <c r="H69" t="n">
-        <v>49</v>
-      </c>
-      <c r="I69" t="n">
-        <v>44.7</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Tata AIA</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Equity - Index (Sector Leaders)</t>
-        </is>
-      </c>
-      <c r="D70" t="n">
-        <v>19</v>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Sector Leaders Index Fund</t>
-        </is>
-      </c>
-      <c r="F70" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="G70" t="n">
-        <v>100</v>
-      </c>
-      <c r="H70" t="n">
-        <v>39</v>
-      </c>
-      <c r="I70" t="n">
-        <v>43.92</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Tata AIA</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Balanced - Debt Oriented</t>
-        </is>
-      </c>
-      <c r="D71" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Whole Life Stable Growth Fund</t>
-        </is>
-      </c>
-      <c r="F71" t="n">
-        <v>100</v>
-      </c>
-      <c r="G71" t="n">
-        <v>100</v>
-      </c>
-      <c r="H71" t="n">
-        <v>64.67</v>
-      </c>
-      <c r="I71" t="n">
         <v>89.40000000000001</v>
       </c>
     </row>

</xml_diff>